<commit_message>
Release 0.4.2: weighted total progress, Earned/Remaining rows
The Total row's progress was a plain average, so a 2-day task counted
as much as a 10-day one. It is now an Excel formula weighted by
time_estimate (SUMPRODUCT / SUMIF), and the estimate total is a SUM, so
both update when the workbook is edited. Blank progress counts as 0 %.

Add optional Earned hours / Remaining hours rows below the Total row,
with short descriptions, in white text by default (GanttStyle.summary_fg,
earned_label/_note, remaining_label/_note).
</commit_message>
<xml_diff>
--- a/examples/bakery-plan.xlsx
+++ b/examples/bakery-plan.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,6 +72,17 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="13">
@@ -177,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -237,6 +248,15 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -634,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX16"/>
+  <dimension ref="A1:AX19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2065,11 +2085,13 @@
         </is>
       </c>
       <c r="B16" s="27" t="n"/>
-      <c r="C16" s="28" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" s="28" t="n">
-        <v>35</v>
+      <c r="C16" s="28">
+        <f>SUM(C4:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="28">
+        <f>IFERROR(ROUND(SUMPRODUCT(C4:C15,D4:D15)/SUMIF(C4:C15,"&gt;0"),1),IFERROR(ROUND(AVERAGE(D4:D15),1),""))</f>
+        <v/>
       </c>
       <c r="E16" s="12" t="n"/>
       <c r="F16" s="12" t="n"/>
@@ -2118,6 +2140,38 @@
       <c r="AW16" s="12" t="n"/>
       <c r="AX16" s="12" t="n"/>
     </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Earned hours</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Time estimate × progress, summed</t>
+        </is>
+      </c>
+      <c r="C18" s="31">
+        <f>ROUND(SUMPRODUCT(C4:C15,D4:D15)/100,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Remaining hours</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Total time estimate − earned</t>
+        </is>
+      </c>
+      <c r="C19" s="31">
+        <f>C16-C18</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:D16"/>
   <mergeCells count="17">
@@ -2148,7 +2202,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3B}">
-          <x14:id>{63B737D6-036E-42B1-88D3-B3875FDABBBA}</x14:id>
+          <x14:id>{3854EFF2-80E3-4B35-8AF2-A9B77CF052E8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2159,7 +2213,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{63B737D6-036E-42B1-88D3-B3875FDABBBA}">
+          <x14:cfRule type="dataBar" id="{3854EFF2-80E3-4B35-8AF2-A9B77CF052E8}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>